<commit_message>
Alinear CA1-CA4 al texto oficial enviado por el profesor
Reemplaza la reformulacion propia de CA1-CA4 (README seccion 7) por la
redaccion oficial del profesor (mensaje del 23/09/2026), y agrega el
campo ca_texto_oficial en artifacts/registry.yaml y en el bloque
trace-data del prototipo para que tools/build_matrix.py lo incluya
tambien en la columna de notas de la matriz generada.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/matriz_trazabilidad_dietas_al_dia.xlsx
+++ b/docs/matriz_trazabilidad_dietas_al_dia.xlsx
@@ -2610,7 +2610,11 @@
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="R4" s="38" t="inlineStr"/>
+      <c r="R4" s="38" t="inlineStr">
+        <is>
+          <t>CA oficial: "Dado un paciente con una enfermedad registrada, el sistema muestra las dietas asociadas en un único paso."</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="24" customHeight="1" s="36">
       <c r="A5" s="12" t="inlineStr">
@@ -2698,7 +2702,11 @@
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="R5" s="2" t="inlineStr"/>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>CA oficial: "Si una dieta recomendada incluye un alimento alérgeno/incompatible del paciente, el sistema lo señala de forma inequívoca antes de confirmar."</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="24" customHeight="1" s="36">
       <c r="A6" s="8" t="inlineStr">
@@ -2786,7 +2794,11 @@
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="R6" s="38" t="inlineStr"/>
+      <c r="R6" s="38" t="inlineStr">
+        <is>
+          <t>CA oficial: "Si una dieta recomendada incluye un alimento alérgeno/incompatible del paciente, el sistema lo señala de forma inequívoca antes de confirmar."</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="24" customHeight="1" s="36">
       <c r="A7" s="12" t="inlineStr">
@@ -2874,7 +2886,11 @@
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="R7" s="2" t="inlineStr"/>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>CA oficial: "El médico accede a la ficha técnica completa de la dieta sin perder el contexto del paciente."</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="24" customHeight="1" s="36">
       <c r="A8" s="8" t="inlineStr">
@@ -2964,7 +2980,7 @@
       </c>
       <c r="R8" s="38" t="inlineStr">
         <is>
-          <t>4 de 5 pruebas de aceptación cumplieron (80 %). Pendiente repetir con un participante adicional tras corregir DEF-05 y DEF-06.</t>
+          <t>CA oficial: "Un usuario nuevo elige una dieta segura en menos de 90 segundos sin pasar por alto ninguna alerta." 4 de 5 pruebas de aceptación cumplieron (80 %). Pendiente repetir con un participante adicional tras corregir DEF-05 y DEF-06.</t>
         </is>
       </c>
     </row>

</xml_diff>